<commit_message>
Add local deployment docs, DB backup, session logs, and update daily summary script
- LOCAL-DEPLOYMENT-INFO.md: Detailed local PostgreSQL setup procedure
- backend/db_backup_2026-01-30.sql: Database backup with users, groups, roles, corpora
- cascade-logs/2026-01-30/: Session documentation and environment resources
- cascade-logs/2026-02-02/: New session summary for Feb 2
- scripts/create-daily-summary.sh: Updated to embed template and use PWD
- Permission-Matrix.xlsx: Updated access control matrix
- Removed deprecated SQLite connection backup file
</commit_message>
<xml_diff>
--- a/Permission-Matrix.xlsx
+++ b/Permission-Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hector/github.com/xtreamgit/adk-multi-agents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7A88A8-67FC-0E42-9B81-D16BAC91D935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455F3EE9-7F2C-8542-926F-008F14A43874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24500" yWindow="2200" windowWidth="32080" windowHeight="27260" xr2:uid="{521A00B9-E13A-2F41-A0C0-6C79EDC12E1F}"/>
+    <workbookView minimized="1" xWindow="7040" yWindow="500" windowWidth="28800" windowHeight="20840" xr2:uid="{521A00B9-E13A-2F41-A0C0-6C79EDC12E1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="161">
   <si>
     <t>admins</t>
   </si>
@@ -109,12 +109,6 @@
   </si>
   <si>
     <t>Agents</t>
-  </si>
-  <si>
-    <t>report_generator</t>
-  </si>
-  <si>
-    <t>queries_only</t>
   </si>
   <si>
     <t>Financial &amp; Accounting Corpora</t>
@@ -510,6 +504,42 @@
   </si>
   <si>
     <t>New Tools</t>
+  </si>
+  <si>
+    <t>Code Tools</t>
+  </si>
+  <si>
+    <t>add_data.py</t>
+  </si>
+  <si>
+    <t>browse_documents.py</t>
+  </si>
+  <si>
+    <t>create_corpus.py</t>
+  </si>
+  <si>
+    <t>delete_corpus.py</t>
+  </si>
+  <si>
+    <t>delete_document.py</t>
+  </si>
+  <si>
+    <t>get_corpus_info.py</t>
+  </si>
+  <si>
+    <t>list_corpora.py</t>
+  </si>
+  <si>
+    <t>rag_multi_query.py</t>
+  </si>
+  <si>
+    <t>rag_query.py</t>
+  </si>
+  <si>
+    <t>utils.py*</t>
+  </si>
+  <si>
+    <t>not accessed by the users.</t>
   </si>
 </sst>
 </file>
@@ -596,7 +626,7 @@
       <name val="Aptos"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -612,6 +642,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -637,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -696,6 +732,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1038,9 +1077,11 @@
     <col min="2" max="2" width="25.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="12" style="3" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="10" style="3" customWidth="1"/>
+    <col min="5" max="5" width="2" style="3" customWidth="1"/>
     <col min="6" max="6" width="31.6640625" style="3" customWidth="1"/>
-    <col min="7" max="10" width="18.1640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="33.5" style="3" customWidth="1"/>
+    <col min="8" max="8" width="31.5" style="3" customWidth="1"/>
+    <col min="9" max="10" width="18.1640625" style="3" customWidth="1"/>
     <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -1125,112 +1166,202 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="2" t="s">
+    <row r="19" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C19" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="F19" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="2">
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="21" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E20" s="2"/>
+      <c r="F20" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="2">
         <v>2</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="E21" s="2"/>
+      <c r="F21" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="22" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C22" s="2">
         <v>3</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="23" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="2">
         <v>4</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="3:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="2">
         <v>5</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C25" s="2">
         <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C26" s="2">
         <v>7</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C27" s="2">
         <v>8</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="28" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C29" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="30" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D30" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D31" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="32" spans="3:6" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="D27" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H27" s="1"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C28" s="2">
+        <v>9</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="3:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C29" s="2">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="1"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="3:10" ht="43" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G30" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="3:10" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="3:10" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="33" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" ht="43" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -1255,7 +1386,7 @@
   <sheetData>
     <row r="2" spans="2:8" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -1266,7 +1397,7 @@
     </row>
     <row r="3" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -1277,10 +1408,10 @@
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>14</v>
@@ -1288,435 +1419,435 @@
     </row>
     <row r="5" spans="2:8" ht="38" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C5" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G5" s="9"/>
     </row>
     <row r="6" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D6" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D7" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D8" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C10" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="2:8" s="4" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D11" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="2:8" s="4" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="2:8" s="4" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D13" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="2:8" s="4" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D14" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" spans="2:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D16" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D18" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D19" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D21" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D22" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D23" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C25" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D26" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D27" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D28" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D29" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C30" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F30" s="10"/>
     </row>
     <row r="31" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D31" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D32" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F32" s="20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D33" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D34" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C35" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D36" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D37" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D38" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="3:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D39" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>